<commit_message>
feat: frontend fix states for user upload
</commit_message>
<xml_diff>
--- a/files/users.xlsx
+++ b/files/users.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/zanbedrac/projects/fitcode/files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{27043D14-D40C-974F-8DEA-8786856AB449}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3463A058-DA25-004A-A16E-F1F2FE9D1110}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17420" xr2:uid="{F61A7227-E63E-E64D-860A-8FA539F3DD59}"/>
+    <workbookView xWindow="-28800" yWindow="580" windowWidth="28800" windowHeight="17420" xr2:uid="{F61A7227-E63E-E64D-860A-8FA539F3DD59}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="57">
   <si>
     <t>displayName</t>
   </si>
@@ -180,6 +180,33 @@
   </si>
   <si>
     <t>athlete</t>
+  </si>
+  <si>
+    <t>sport</t>
+  </si>
+  <si>
+    <t>level</t>
+  </si>
+  <si>
+    <t>gender</t>
+  </si>
+  <si>
+    <t>birthDate</t>
+  </si>
+  <si>
+    <t>intermediate</t>
+  </si>
+  <si>
+    <t>beginner</t>
+  </si>
+  <si>
+    <t>advanced</t>
+  </si>
+  <si>
+    <t>male</t>
+  </si>
+  <si>
+    <t>Football</t>
   </si>
 </sst>
 </file>
@@ -245,12 +272,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -586,24 +614,26 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{97433651-90B5-E649-8E0D-B1555FFB3972}">
-  <dimension ref="A1:E16"/>
+  <dimension ref="A1:I16"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="35.83203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="27.83203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.1640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="27.83203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.1640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="35.83203125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="46.5" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.6640625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="9" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A1" s="2" t="s">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>0</v>
-      </c>
-      <c r="B1" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="3" t="s">
-        <v>2</v>
       </c>
       <c r="D1" s="3" t="s">
         <v>3</v>
@@ -611,16 +641,28 @@
       <c r="E1" s="3" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A2" s="1" t="s">
+      <c r="F1" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="I1" s="3" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A2" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="B2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C2" s="1" t="s">
         <v>4</v>
-      </c>
-      <c r="B2" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="C2" t="s">
-        <v>2</v>
       </c>
       <c r="D2" t="s">
         <v>32</v>
@@ -628,16 +670,28 @@
       <c r="E2" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A3" s="1" t="s">
+      <c r="F2" t="s">
+        <v>56</v>
+      </c>
+      <c r="G2" t="s">
+        <v>52</v>
+      </c>
+      <c r="H2" t="s">
+        <v>55</v>
+      </c>
+      <c r="I2" s="5">
+        <v>38849</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A3" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="B3" t="s">
+        <v>2</v>
+      </c>
+      <c r="C3" s="1" t="s">
         <v>5</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="C3" t="s">
-        <v>2</v>
       </c>
       <c r="D3" t="s">
         <v>33</v>
@@ -645,16 +699,28 @@
       <c r="E3" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A4" s="1" t="s">
+      <c r="F3" t="s">
+        <v>56</v>
+      </c>
+      <c r="G3" t="s">
+        <v>53</v>
+      </c>
+      <c r="H3" t="s">
+        <v>55</v>
+      </c>
+      <c r="I3" s="5">
+        <v>38850</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A4" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B4" t="s">
+        <v>2</v>
+      </c>
+      <c r="C4" s="1" t="s">
         <v>6</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="C4" t="s">
-        <v>2</v>
       </c>
       <c r="D4" t="s">
         <v>34</v>
@@ -662,16 +728,28 @@
       <c r="E4" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A5" s="1" t="s">
+      <c r="F4" t="s">
+        <v>56</v>
+      </c>
+      <c r="G4" t="s">
+        <v>54</v>
+      </c>
+      <c r="H4" t="s">
+        <v>55</v>
+      </c>
+      <c r="I4" s="5">
+        <v>38851</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A5" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="B5" t="s">
+        <v>2</v>
+      </c>
+      <c r="C5" s="1" t="s">
         <v>7</v>
-      </c>
-      <c r="B5" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="C5" t="s">
-        <v>2</v>
       </c>
       <c r="D5" t="s">
         <v>35</v>
@@ -679,16 +757,28 @@
       <c r="E5" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A6" s="1" t="s">
+      <c r="F5" t="s">
+        <v>56</v>
+      </c>
+      <c r="G5" t="s">
+        <v>52</v>
+      </c>
+      <c r="H5" t="s">
+        <v>55</v>
+      </c>
+      <c r="I5" s="5">
+        <v>38852</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A6" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="B6" t="s">
+        <v>2</v>
+      </c>
+      <c r="C6" s="1" t="s">
         <v>8</v>
-      </c>
-      <c r="B6" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="C6" t="s">
-        <v>2</v>
       </c>
       <c r="D6" t="s">
         <v>36</v>
@@ -696,16 +786,28 @@
       <c r="E6" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A7" s="1" t="s">
+      <c r="F6" t="s">
+        <v>56</v>
+      </c>
+      <c r="G6" t="s">
+        <v>52</v>
+      </c>
+      <c r="H6" t="s">
+        <v>55</v>
+      </c>
+      <c r="I6" s="5">
+        <v>38853</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A7" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="B7" t="s">
+        <v>2</v>
+      </c>
+      <c r="C7" s="1" t="s">
         <v>9</v>
-      </c>
-      <c r="B7" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="C7" t="s">
-        <v>2</v>
       </c>
       <c r="D7" t="s">
         <v>37</v>
@@ -713,16 +815,28 @@
       <c r="E7" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A8" s="1" t="s">
+      <c r="F7" t="s">
+        <v>56</v>
+      </c>
+      <c r="G7" t="s">
+        <v>52</v>
+      </c>
+      <c r="H7" t="s">
+        <v>55</v>
+      </c>
+      <c r="I7" s="5">
+        <v>38854</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A8" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="B8" t="s">
+        <v>2</v>
+      </c>
+      <c r="C8" s="1" t="s">
         <v>10</v>
-      </c>
-      <c r="B8" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="C8" t="s">
-        <v>2</v>
       </c>
       <c r="D8" t="s">
         <v>38</v>
@@ -730,16 +844,28 @@
       <c r="E8" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A9" s="1" t="s">
+      <c r="F8" t="s">
+        <v>56</v>
+      </c>
+      <c r="G8" t="s">
+        <v>52</v>
+      </c>
+      <c r="H8" t="s">
+        <v>55</v>
+      </c>
+      <c r="I8" s="5">
+        <v>38855</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A9" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="B9" t="s">
+        <v>2</v>
+      </c>
+      <c r="C9" s="1" t="s">
         <v>11</v>
-      </c>
-      <c r="B9" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="C9" t="s">
-        <v>2</v>
       </c>
       <c r="D9" t="s">
         <v>39</v>
@@ -747,16 +873,28 @@
       <c r="E9" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A10" s="1" t="s">
+      <c r="F9" t="s">
+        <v>56</v>
+      </c>
+      <c r="G9" t="s">
+        <v>52</v>
+      </c>
+      <c r="H9" t="s">
+        <v>55</v>
+      </c>
+      <c r="I9" s="5">
+        <v>38856</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A10" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B10" t="s">
+        <v>2</v>
+      </c>
+      <c r="C10" s="1" t="s">
         <v>12</v>
-      </c>
-      <c r="B10" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="C10" t="s">
-        <v>2</v>
       </c>
       <c r="D10" t="s">
         <v>40</v>
@@ -764,16 +902,28 @@
       <c r="E10" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A11" s="1" t="s">
+      <c r="F10" t="s">
+        <v>56</v>
+      </c>
+      <c r="G10" t="s">
+        <v>52</v>
+      </c>
+      <c r="H10" t="s">
+        <v>55</v>
+      </c>
+      <c r="I10" s="5">
+        <v>38857</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A11" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="B11" t="s">
+        <v>2</v>
+      </c>
+      <c r="C11" s="1" t="s">
         <v>13</v>
-      </c>
-      <c r="B11" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="C11" t="s">
-        <v>2</v>
       </c>
       <c r="D11" t="s">
         <v>41</v>
@@ -781,16 +931,28 @@
       <c r="E11" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A12" s="1" t="s">
+      <c r="F11" t="s">
+        <v>56</v>
+      </c>
+      <c r="G11" t="s">
+        <v>52</v>
+      </c>
+      <c r="H11" t="s">
+        <v>55</v>
+      </c>
+      <c r="I11" s="5">
+        <v>38858</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A12" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="B12" t="s">
+        <v>2</v>
+      </c>
+      <c r="C12" s="1" t="s">
         <v>14</v>
-      </c>
-      <c r="B12" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="C12" t="s">
-        <v>2</v>
       </c>
       <c r="D12" t="s">
         <v>42</v>
@@ -798,16 +960,28 @@
       <c r="E12" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A13" s="1" t="s">
+      <c r="F12" t="s">
+        <v>56</v>
+      </c>
+      <c r="G12" t="s">
+        <v>52</v>
+      </c>
+      <c r="H12" t="s">
+        <v>55</v>
+      </c>
+      <c r="I12" s="5">
+        <v>38859</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A13" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="B13" t="s">
+        <v>2</v>
+      </c>
+      <c r="C13" s="1" t="s">
         <v>15</v>
-      </c>
-      <c r="B13" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="C13" t="s">
-        <v>2</v>
       </c>
       <c r="D13" t="s">
         <v>43</v>
@@ -815,16 +989,28 @@
       <c r="E13" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A14" s="1" t="s">
+      <c r="F13" t="s">
+        <v>56</v>
+      </c>
+      <c r="G13" t="s">
+        <v>52</v>
+      </c>
+      <c r="H13" t="s">
+        <v>55</v>
+      </c>
+      <c r="I13" s="5">
+        <v>38860</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A14" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="B14" t="s">
+        <v>2</v>
+      </c>
+      <c r="C14" s="1" t="s">
         <v>16</v>
-      </c>
-      <c r="B14" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="C14" t="s">
-        <v>2</v>
       </c>
       <c r="D14" t="s">
         <v>44</v>
@@ -832,16 +1018,28 @@
       <c r="E14" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A15" s="1" t="s">
+      <c r="F14" t="s">
+        <v>56</v>
+      </c>
+      <c r="G14" t="s">
+        <v>52</v>
+      </c>
+      <c r="H14" t="s">
+        <v>55</v>
+      </c>
+      <c r="I14" s="5">
+        <v>38861</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A15" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="B15" t="s">
+        <v>2</v>
+      </c>
+      <c r="C15" s="1" t="s">
         <v>17</v>
-      </c>
-      <c r="B15" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="C15" t="s">
-        <v>2</v>
       </c>
       <c r="D15" t="s">
         <v>45</v>
@@ -849,26 +1047,38 @@
       <c r="E15" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A16" s="1"/>
+      <c r="F15" t="s">
+        <v>56</v>
+      </c>
+      <c r="G15" t="s">
+        <v>52</v>
+      </c>
+      <c r="H15" t="s">
+        <v>55</v>
+      </c>
+      <c r="I15" s="5">
+        <v>38862</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="C16" s="1"/>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="B2" r:id="rId1" xr:uid="{489300CC-9BC2-3F43-AB39-3EEB8054079D}"/>
-    <hyperlink ref="B3" r:id="rId2" xr:uid="{A92ABC1A-88FB-274B-9086-1D5409849BAF}"/>
-    <hyperlink ref="B4" r:id="rId3" xr:uid="{58939A25-AD0F-3A4D-969C-DCC750A979E0}"/>
-    <hyperlink ref="B5" r:id="rId4" xr:uid="{D2F1DD65-8225-FC4E-AA47-FD892FEB1AC5}"/>
-    <hyperlink ref="B6" r:id="rId5" xr:uid="{1B04BBFD-0C09-0249-8A29-E251F14CDD1F}"/>
-    <hyperlink ref="B7" r:id="rId6" xr:uid="{EA971285-93ED-0041-AA6F-B4CB066F5F53}"/>
-    <hyperlink ref="B8" r:id="rId7" xr:uid="{774F915E-7B60-ED40-9B79-35B680F73B31}"/>
-    <hyperlink ref="B9" r:id="rId8" xr:uid="{11F47E88-3EA5-0E41-B726-22B8214101A0}"/>
-    <hyperlink ref="B10" r:id="rId9" xr:uid="{B4A78F48-D0E6-784E-8FF0-93EA2E6CC30D}"/>
-    <hyperlink ref="B11" r:id="rId10" xr:uid="{07ED519C-F5EA-4745-8007-132251FDE1A1}"/>
-    <hyperlink ref="B12" r:id="rId11" xr:uid="{9F6ABA26-AB0F-3B44-8B22-DCAD133D0816}"/>
-    <hyperlink ref="B13" r:id="rId12" xr:uid="{7428667B-492C-E74C-828F-155A3454DFFB}"/>
-    <hyperlink ref="B14" r:id="rId13" xr:uid="{E51A0C12-7F5B-3E40-9B8F-571D842A5D98}"/>
-    <hyperlink ref="B15" r:id="rId14" xr:uid="{84ACF764-9124-7C44-A536-331B558FCC18}"/>
+    <hyperlink ref="A2" r:id="rId1" xr:uid="{489300CC-9BC2-3F43-AB39-3EEB8054079D}"/>
+    <hyperlink ref="A3" r:id="rId2" xr:uid="{A92ABC1A-88FB-274B-9086-1D5409849BAF}"/>
+    <hyperlink ref="A4" r:id="rId3" xr:uid="{58939A25-AD0F-3A4D-969C-DCC750A979E0}"/>
+    <hyperlink ref="A5" r:id="rId4" xr:uid="{D2F1DD65-8225-FC4E-AA47-FD892FEB1AC5}"/>
+    <hyperlink ref="A6" r:id="rId5" xr:uid="{1B04BBFD-0C09-0249-8A29-E251F14CDD1F}"/>
+    <hyperlink ref="A7" r:id="rId6" xr:uid="{EA971285-93ED-0041-AA6F-B4CB066F5F53}"/>
+    <hyperlink ref="A8" r:id="rId7" xr:uid="{774F915E-7B60-ED40-9B79-35B680F73B31}"/>
+    <hyperlink ref="A9" r:id="rId8" xr:uid="{11F47E88-3EA5-0E41-B726-22B8214101A0}"/>
+    <hyperlink ref="A10" r:id="rId9" xr:uid="{B4A78F48-D0E6-784E-8FF0-93EA2E6CC30D}"/>
+    <hyperlink ref="A11" r:id="rId10" xr:uid="{07ED519C-F5EA-4745-8007-132251FDE1A1}"/>
+    <hyperlink ref="A12" r:id="rId11" xr:uid="{9F6ABA26-AB0F-3B44-8B22-DCAD133D0816}"/>
+    <hyperlink ref="A13" r:id="rId12" xr:uid="{7428667B-492C-E74C-828F-155A3454DFFB}"/>
+    <hyperlink ref="A14" r:id="rId13" xr:uid="{E51A0C12-7F5B-3E40-9B8F-571D842A5D98}"/>
+    <hyperlink ref="A15" r:id="rId14" xr:uid="{84ACF764-9124-7C44-A536-331B558FCC18}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
refactor: remove firebase functions completely and replace with custom backend route calls
</commit_message>
<xml_diff>
--- a/files/users.xlsx
+++ b/files/users.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/zanbedrac/projects/fitcode/files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3463A058-DA25-004A-A16E-F1F2FE9D1110}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2F0F2CD1-5B8F-8C42-A896-D7B2D148D016}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28800" yWindow="580" windowWidth="28800" windowHeight="17420" xr2:uid="{F61A7227-E63E-E64D-860A-8FA539F3DD59}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17420" xr2:uid="{F61A7227-E63E-E64D-860A-8FA539F3DD59}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="61">
   <si>
     <t>displayName</t>
   </si>
@@ -207,6 +207,18 @@
   </si>
   <si>
     <t>Football</t>
+  </si>
+  <si>
+    <t>tomi.jagarinec@mail.com</t>
+  </si>
+  <si>
+    <t>Tomi Jagarinec</t>
+  </si>
+  <si>
+    <t>https://iamaspire.aspire.qa/assets/Tomaz.png</t>
+  </si>
+  <si>
+    <t>trainer</t>
   </si>
 </sst>
 </file>
@@ -272,13 +284,15 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -614,7 +628,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{97433651-90B5-E649-8E0D-B1555FFB3972}">
-  <dimension ref="A1:I16"/>
+  <dimension ref="A1:I17"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="27.83203125" bestFit="1" customWidth="1"/>
@@ -654,47 +668,47 @@
         <v>51</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:9" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A2" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="B2" t="s">
+        <v>57</v>
+      </c>
+      <c r="B2" s="6" t="s">
         <v>2</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="D2" t="s">
-        <v>32</v>
-      </c>
-      <c r="E2" t="s">
-        <v>47</v>
-      </c>
-      <c r="F2" t="s">
-        <v>56</v>
-      </c>
-      <c r="G2" t="s">
-        <v>52</v>
-      </c>
-      <c r="H2" t="s">
-        <v>55</v>
-      </c>
-      <c r="I2" s="5">
-        <v>38849</v>
+        <v>58</v>
+      </c>
+      <c r="D2" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="E2" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="F2" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="G2" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="H2" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="I2" s="7">
+        <v>29531</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A3" s="4" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B3" t="s">
         <v>2</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E3" t="s">
         <v>47</v>
@@ -703,27 +717,27 @@
         <v>56</v>
       </c>
       <c r="G3" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="H3" t="s">
         <v>55</v>
       </c>
       <c r="I3" s="5">
-        <v>38850</v>
+        <v>38849</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A4" s="4" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B4" t="s">
         <v>2</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D4" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E4" t="s">
         <v>47</v>
@@ -732,27 +746,27 @@
         <v>56</v>
       </c>
       <c r="G4" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="H4" t="s">
         <v>55</v>
       </c>
       <c r="I4" s="5">
-        <v>38851</v>
+        <v>38850</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A5" s="4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B5" t="s">
         <v>2</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D5" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E5" t="s">
         <v>47</v>
@@ -761,27 +775,27 @@
         <v>56</v>
       </c>
       <c r="G5" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="H5" t="s">
         <v>55</v>
       </c>
       <c r="I5" s="5">
-        <v>38852</v>
+        <v>38851</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A6" s="4" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B6" t="s">
         <v>2</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D6" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E6" t="s">
         <v>47</v>
@@ -796,21 +810,21 @@
         <v>55</v>
       </c>
       <c r="I6" s="5">
-        <v>38853</v>
+        <v>38852</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A7" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B7" t="s">
         <v>2</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D7" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E7" t="s">
         <v>47</v>
@@ -825,21 +839,21 @@
         <v>55</v>
       </c>
       <c r="I7" s="5">
-        <v>38854</v>
+        <v>38853</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A8" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B8" t="s">
         <v>2</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D8" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E8" t="s">
         <v>47</v>
@@ -854,21 +868,21 @@
         <v>55</v>
       </c>
       <c r="I8" s="5">
-        <v>38855</v>
+        <v>38854</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A9" s="4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B9" t="s">
         <v>2</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D9" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E9" t="s">
         <v>47</v>
@@ -883,21 +897,21 @@
         <v>55</v>
       </c>
       <c r="I9" s="5">
-        <v>38856</v>
+        <v>38855</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A10" s="4" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B10" t="s">
         <v>2</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D10" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E10" t="s">
         <v>47</v>
@@ -912,21 +926,21 @@
         <v>55</v>
       </c>
       <c r="I10" s="5">
-        <v>38857</v>
+        <v>38856</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A11" s="4" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B11" t="s">
         <v>2</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D11" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E11" t="s">
         <v>47</v>
@@ -941,21 +955,21 @@
         <v>55</v>
       </c>
       <c r="I11" s="5">
-        <v>38858</v>
+        <v>38857</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A12" s="4" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B12" t="s">
         <v>2</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D12" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E12" t="s">
         <v>47</v>
@@ -970,21 +984,21 @@
         <v>55</v>
       </c>
       <c r="I12" s="5">
-        <v>38859</v>
+        <v>38858</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A13" s="4" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B13" t="s">
         <v>2</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D13" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E13" t="s">
         <v>47</v>
@@ -999,21 +1013,21 @@
         <v>55</v>
       </c>
       <c r="I13" s="5">
-        <v>38860</v>
+        <v>38859</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A14" s="4" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B14" t="s">
         <v>2</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D14" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E14" t="s">
         <v>47</v>
@@ -1028,21 +1042,21 @@
         <v>55</v>
       </c>
       <c r="I14" s="5">
-        <v>38861</v>
+        <v>38860</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A15" s="4" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B15" t="s">
         <v>2</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D15" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E15" t="s">
         <v>47</v>
@@ -1057,28 +1071,58 @@
         <v>55</v>
       </c>
       <c r="I15" s="5">
+        <v>38861</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A16" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="B16" t="s">
+        <v>2</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D16" t="s">
+        <v>45</v>
+      </c>
+      <c r="E16" t="s">
+        <v>47</v>
+      </c>
+      <c r="F16" t="s">
+        <v>56</v>
+      </c>
+      <c r="G16" t="s">
+        <v>52</v>
+      </c>
+      <c r="H16" t="s">
+        <v>55</v>
+      </c>
+      <c r="I16" s="5">
         <v>38862</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="C16" s="1"/>
+    <row r="17" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C17" s="1"/>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="A2" r:id="rId1" xr:uid="{489300CC-9BC2-3F43-AB39-3EEB8054079D}"/>
-    <hyperlink ref="A3" r:id="rId2" xr:uid="{A92ABC1A-88FB-274B-9086-1D5409849BAF}"/>
-    <hyperlink ref="A4" r:id="rId3" xr:uid="{58939A25-AD0F-3A4D-969C-DCC750A979E0}"/>
-    <hyperlink ref="A5" r:id="rId4" xr:uid="{D2F1DD65-8225-FC4E-AA47-FD892FEB1AC5}"/>
-    <hyperlink ref="A6" r:id="rId5" xr:uid="{1B04BBFD-0C09-0249-8A29-E251F14CDD1F}"/>
-    <hyperlink ref="A7" r:id="rId6" xr:uid="{EA971285-93ED-0041-AA6F-B4CB066F5F53}"/>
-    <hyperlink ref="A8" r:id="rId7" xr:uid="{774F915E-7B60-ED40-9B79-35B680F73B31}"/>
-    <hyperlink ref="A9" r:id="rId8" xr:uid="{11F47E88-3EA5-0E41-B726-22B8214101A0}"/>
-    <hyperlink ref="A10" r:id="rId9" xr:uid="{B4A78F48-D0E6-784E-8FF0-93EA2E6CC30D}"/>
-    <hyperlink ref="A11" r:id="rId10" xr:uid="{07ED519C-F5EA-4745-8007-132251FDE1A1}"/>
-    <hyperlink ref="A12" r:id="rId11" xr:uid="{9F6ABA26-AB0F-3B44-8B22-DCAD133D0816}"/>
-    <hyperlink ref="A13" r:id="rId12" xr:uid="{7428667B-492C-E74C-828F-155A3454DFFB}"/>
-    <hyperlink ref="A14" r:id="rId13" xr:uid="{E51A0C12-7F5B-3E40-9B8F-571D842A5D98}"/>
-    <hyperlink ref="A15" r:id="rId14" xr:uid="{84ACF764-9124-7C44-A536-331B558FCC18}"/>
+    <hyperlink ref="A3" r:id="rId1" xr:uid="{489300CC-9BC2-3F43-AB39-3EEB8054079D}"/>
+    <hyperlink ref="A4" r:id="rId2" xr:uid="{A92ABC1A-88FB-274B-9086-1D5409849BAF}"/>
+    <hyperlink ref="A5" r:id="rId3" xr:uid="{58939A25-AD0F-3A4D-969C-DCC750A979E0}"/>
+    <hyperlink ref="A6" r:id="rId4" xr:uid="{D2F1DD65-8225-FC4E-AA47-FD892FEB1AC5}"/>
+    <hyperlink ref="A7" r:id="rId5" xr:uid="{1B04BBFD-0C09-0249-8A29-E251F14CDD1F}"/>
+    <hyperlink ref="A8" r:id="rId6" xr:uid="{EA971285-93ED-0041-AA6F-B4CB066F5F53}"/>
+    <hyperlink ref="A9" r:id="rId7" xr:uid="{774F915E-7B60-ED40-9B79-35B680F73B31}"/>
+    <hyperlink ref="A10" r:id="rId8" xr:uid="{11F47E88-3EA5-0E41-B726-22B8214101A0}"/>
+    <hyperlink ref="A11" r:id="rId9" xr:uid="{B4A78F48-D0E6-784E-8FF0-93EA2E6CC30D}"/>
+    <hyperlink ref="A12" r:id="rId10" xr:uid="{07ED519C-F5EA-4745-8007-132251FDE1A1}"/>
+    <hyperlink ref="A13" r:id="rId11" xr:uid="{9F6ABA26-AB0F-3B44-8B22-DCAD133D0816}"/>
+    <hyperlink ref="A14" r:id="rId12" xr:uid="{7428667B-492C-E74C-828F-155A3454DFFB}"/>
+    <hyperlink ref="A15" r:id="rId13" xr:uid="{E51A0C12-7F5B-3E40-9B8F-571D842A5D98}"/>
+    <hyperlink ref="A16" r:id="rId14" xr:uid="{84ACF764-9124-7C44-A536-331B558FCC18}"/>
+    <hyperlink ref="A2" r:id="rId15" xr:uid="{3CCFB96D-6543-E249-B94D-CF33859BD697}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>